<commit_message>
remove README and Methodology tabs from workbook, checked by Cole
</commit_message>
<xml_diff>
--- a/outputs/camera_analysis_results.xlsx
+++ b/outputs/camera_analysis_results.xlsx
@@ -7,11 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Per_Camera" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Placebo" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Methodology" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Per_Camera" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Placebo" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,22 +21,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F3A5F"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -49,20 +38,6 @@
     <font>
       <b val="1"/>
       <sz val="13"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="15"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="12"/>
     </font>
   </fonts>
   <fills count="6">
@@ -105,27 +80,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -491,123 +455,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>DC Traffic Camera Impact Analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Analysis window: crash data from 2021 through 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Eligible cameras: 283 live cameras with a full 365-day pre and post window.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Buffer: 200m radius around each camera (roughly two DC blocks).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Primary metric: Difference-in-Differences (DiD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  = (nearby % change) minus (citywide % change)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Negative DiD = area near camera improved MORE than citywide trend.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Positive DiD = area near camera improved LESS than citywide trend.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TABS:</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Summary      — Headline DiD by camera type and outcome</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Per_Camera   — One row per camera, all computed columns</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Placebo      — Real DiD vs placebo DiD (install shifted back 1 yr)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Methodology  — Design notes and caveats</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -624,7 +471,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Headline results by camera type — 200m buffer</t>
         </is>
@@ -632,52 +479,52 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Camera Type</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Outcome</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Nearby pre</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Nearby post</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Nearby %</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Citywide %</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>DiD</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Placebo DiD</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Corrected DiD (Real - Placebo)</t>
         </is>
@@ -709,7 +556,7 @@
       <c r="G4" t="n">
         <v>-4.4</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="H4" s="3" t="n">
         <v>0.8</v>
       </c>
       <c r="I4" t="n">
@@ -745,7 +592,7 @@
       <c r="G5" t="n">
         <v>-5.9</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="3" t="n">
         <v>1.9</v>
       </c>
       <c r="I5" t="n">
@@ -781,7 +628,7 @@
       <c r="G6" t="n">
         <v>-2.9</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="H6" s="4" t="n">
         <v>-7.8</v>
       </c>
       <c r="I6" t="n">
@@ -817,7 +664,7 @@
       <c r="G7" t="n">
         <v>-5.4</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="H7" s="4" t="n">
         <v>-5.2</v>
       </c>
       <c r="I7" t="n">
@@ -854,7 +701,7 @@
       <c r="G9" t="n">
         <v>-5</v>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="H9" s="5" t="n">
         <v>6.7</v>
       </c>
       <c r="I9" t="n">
@@ -890,7 +737,7 @@
       <c r="G10" t="n">
         <v>-6.2</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="3" t="n">
         <v>2.3</v>
       </c>
       <c r="I10" t="n">
@@ -926,7 +773,7 @@
       <c r="G11" t="n">
         <v>-3.2</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="H11" s="4" t="n">
         <v>-17.3</v>
       </c>
       <c r="I11" t="n">
@@ -962,7 +809,7 @@
       <c r="G12" t="n">
         <v>-5.7</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H12" s="4" t="n">
         <v>-15.8</v>
       </c>
       <c r="I12" t="n">
@@ -999,7 +846,7 @@
       <c r="G14" t="n">
         <v>-10.3</v>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="H14" s="3" t="n">
         <v>-4.7</v>
       </c>
       <c r="I14" t="n">
@@ -1035,7 +882,7 @@
       <c r="G15" t="n">
         <v>-10.4</v>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="H15" s="5" t="n">
         <v>27.9</v>
       </c>
       <c r="I15" t="n">
@@ -1071,7 +918,7 @@
       <c r="G16" t="n">
         <v>-7.6</v>
       </c>
-      <c r="H16" s="7" t="n">
+      <c r="H16" s="5" t="n">
         <v>27.6</v>
       </c>
       <c r="I16" t="n">
@@ -1107,7 +954,7 @@
       <c r="G17" t="n">
         <v>-12.8</v>
       </c>
-      <c r="H17" s="7" t="n">
+      <c r="H17" s="5" t="n">
         <v>12.8</v>
       </c>
       <c r="I17" t="n">
@@ -1144,7 +991,7 @@
       <c r="G19" t="n">
         <v>-1.7</v>
       </c>
-      <c r="H19" s="6" t="n">
+      <c r="H19" s="4" t="n">
         <v>-12.6</v>
       </c>
       <c r="I19" t="n">
@@ -1180,7 +1027,7 @@
       <c r="G20" t="n">
         <v>-9</v>
       </c>
-      <c r="H20" s="6" t="n">
+      <c r="H20" s="4" t="n">
         <v>-31</v>
       </c>
       <c r="I20" t="n">
@@ -1246,7 +1093,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1284,132 +1131,132 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>camera_code</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>install_date</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>ward</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>lat</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>lon</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>nearby_all_pre</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>nearby_all_post</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>nearby_all_pct</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>nearby_injury_pre</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>nearby_injury_post</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>nearby_injury_pct</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>nearby_serious_pre</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>nearby_serious_post</t>
         </is>
       </c>
-      <c r="P1" s="4" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>nearby_serious_pct</t>
         </is>
       </c>
-      <c r="Q1" s="4" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>nearby_fatal_pre</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>nearby_fatal_post</t>
         </is>
       </c>
-      <c r="S1" s="4" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>nearby_fatal_pct</t>
         </is>
       </c>
-      <c r="T1" s="4" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>citywide_all_pct</t>
         </is>
       </c>
-      <c r="U1" s="4" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>citywide_injury_pct</t>
         </is>
       </c>
-      <c r="V1" s="4" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>did_all</t>
         </is>
       </c>
-      <c r="W1" s="4" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>did_injury</t>
         </is>
       </c>
-      <c r="X1" s="4" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>did_serious</t>
         </is>
       </c>
-      <c r="Y1" s="4" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>did_fatal</t>
         </is>
       </c>
-      <c r="Z1" s="4" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>did_speeding</t>
         </is>
@@ -1431,7 +1278,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D2" s="8" t="n">
+      <c r="D2" s="6" t="n">
         <v>45149</v>
       </c>
       <c r="E2" t="n">
@@ -1511,7 +1358,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D3" s="8" t="n">
+      <c r="D3" s="6" t="n">
         <v>45189</v>
       </c>
       <c r="E3" t="n">
@@ -1582,7 +1429,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="6" t="n">
         <v>45277</v>
       </c>
       <c r="E4" t="n">
@@ -1662,7 +1509,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="6" t="n">
         <v>45278</v>
       </c>
       <c r="E5" t="n">
@@ -1742,7 +1589,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="6" t="n">
         <v>45278</v>
       </c>
       <c r="E6" t="n">
@@ -1822,7 +1669,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="6" t="n">
         <v>45278</v>
       </c>
       <c r="E7" t="n">
@@ -1902,7 +1749,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="6" t="n">
         <v>45290</v>
       </c>
       <c r="E8" t="n">
@@ -1982,7 +1829,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="6" t="n">
         <v>45294</v>
       </c>
       <c r="E9" t="n">
@@ -2062,7 +1909,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="6" t="n">
         <v>45305</v>
       </c>
       <c r="E10" t="n">
@@ -2133,7 +1980,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="6" t="n">
         <v>45331</v>
       </c>
       <c r="E11" t="n">
@@ -2207,7 +2054,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="6" t="n">
         <v>45331</v>
       </c>
       <c r="E12" t="n">
@@ -2278,7 +2125,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="6" t="n">
         <v>45364</v>
       </c>
       <c r="E13" t="n">
@@ -2358,7 +2205,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="6" t="n">
         <v>45365</v>
       </c>
       <c r="E14" t="n">
@@ -2444,7 +2291,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="D15" s="6" t="n">
         <v>45398</v>
       </c>
       <c r="E15" t="n">
@@ -2521,7 +2368,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D16" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E16" t="n">
@@ -2598,7 +2445,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D17" s="8" t="n">
+      <c r="D17" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E17" t="n">
@@ -2669,7 +2516,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="D18" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E18" t="n">
@@ -2740,7 +2587,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D19" s="8" t="n">
+      <c r="D19" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E19" t="n">
@@ -2817,7 +2664,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D20" s="8" t="n">
+      <c r="D20" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E20" t="n">
@@ -2894,7 +2741,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D21" s="8" t="n">
+      <c r="D21" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E21" t="n">
@@ -2968,7 +2815,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D22" s="8" t="n">
+      <c r="D22" s="6" t="n">
         <v>45484</v>
       </c>
       <c r="E22" t="n">
@@ -3042,7 +2889,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D23" s="8" t="n">
+      <c r="D23" s="6" t="n">
         <v>45273</v>
       </c>
       <c r="E23" t="n">
@@ -3116,7 +2963,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D24" s="8" t="n">
+      <c r="D24" s="6" t="n">
         <v>45273</v>
       </c>
       <c r="E24" t="n">
@@ -3196,7 +3043,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D25" s="8" t="n">
+      <c r="D25" s="6" t="n">
         <v>45278</v>
       </c>
       <c r="E25" t="n">
@@ -3270,7 +3117,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D26" s="8" t="n">
+      <c r="D26" s="6" t="n">
         <v>45290</v>
       </c>
       <c r="E26" t="n">
@@ -3350,7 +3197,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D27" s="8" t="n">
+      <c r="D27" s="6" t="n">
         <v>45290</v>
       </c>
       <c r="E27" t="n">
@@ -3430,7 +3277,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D28" s="8" t="n">
+      <c r="D28" s="6" t="n">
         <v>45305</v>
       </c>
       <c r="E28" t="n">
@@ -3504,7 +3351,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D29" s="8" t="n">
+      <c r="D29" s="6" t="n">
         <v>45330</v>
       </c>
       <c r="E29" t="n">
@@ -3575,7 +3422,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D30" s="8" t="n">
+      <c r="D30" s="6" t="n">
         <v>45330</v>
       </c>
       <c r="E30" t="n">
@@ -3649,7 +3496,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D31" s="8" t="n">
+      <c r="D31" s="6" t="n">
         <v>45352</v>
       </c>
       <c r="E31" t="n">
@@ -3729,7 +3576,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D32" s="8" t="n">
+      <c r="D32" s="6" t="n">
         <v>45357</v>
       </c>
       <c r="E32" t="n">
@@ -3806,7 +3653,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D33" s="8" t="n">
+      <c r="D33" s="6" t="n">
         <v>45364</v>
       </c>
       <c r="E33" t="n">
@@ -3880,7 +3727,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D34" s="8" t="n">
+      <c r="D34" s="6" t="n">
         <v>45365</v>
       </c>
       <c r="E34" t="n">
@@ -3960,7 +3807,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D35" s="8" t="n">
+      <c r="D35" s="6" t="n">
         <v>45365</v>
       </c>
       <c r="E35" t="n">
@@ -4037,7 +3884,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D36" s="8" t="n">
+      <c r="D36" s="6" t="n">
         <v>45370</v>
       </c>
       <c r="E36" t="n">
@@ -4102,7 +3949,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D37" s="8" t="n">
+      <c r="D37" s="6" t="n">
         <v>45373</v>
       </c>
       <c r="E37" t="n">
@@ -4179,7 +4026,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D38" s="8" t="n">
+      <c r="D38" s="6" t="n">
         <v>45381</v>
       </c>
       <c r="E38" t="n">
@@ -4253,7 +4100,7 @@
           <t>Truck Restriction</t>
         </is>
       </c>
-      <c r="D39" s="8" t="n">
+      <c r="D39" s="6" t="n">
         <v>45383</v>
       </c>
       <c r="E39" t="n">
@@ -4333,7 +4180,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D40" s="8" t="n">
+      <c r="D40" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E40" t="n">
@@ -4413,7 +4260,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D41" s="8" t="n">
+      <c r="D41" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E41" t="n">
@@ -4493,7 +4340,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D42" s="8" t="n">
+      <c r="D42" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E42" t="n">
@@ -4567,7 +4414,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D43" s="8" t="n">
+      <c r="D43" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E43" t="n">
@@ -4644,7 +4491,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D44" s="8" t="n">
+      <c r="D44" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E44" t="n">
@@ -4724,7 +4571,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D45" s="8" t="n">
+      <c r="D45" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E45" t="n">
@@ -4810,7 +4657,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D46" s="8" t="n">
+      <c r="D46" s="6" t="n">
         <v>45412</v>
       </c>
       <c r="E46" t="n">
@@ -4896,7 +4743,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D47" s="8" t="n">
+      <c r="D47" s="6" t="n">
         <v>45426</v>
       </c>
       <c r="E47" t="n">
@@ -4961,7 +4808,7 @@
           <t>Truck Restriction</t>
         </is>
       </c>
-      <c r="D48" s="8" t="n">
+      <c r="D48" s="6" t="n">
         <v>45433</v>
       </c>
       <c r="E48" t="n">
@@ -5035,7 +4882,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D49" s="8" t="n">
+      <c r="D49" s="6" t="n">
         <v>45540</v>
       </c>
       <c r="E49" t="n">
@@ -5106,7 +4953,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D50" s="8" t="n">
+      <c r="D50" s="6" t="n">
         <v>45619</v>
       </c>
       <c r="E50" t="n">
@@ -5186,7 +5033,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D51" s="8" t="n">
+      <c r="D51" s="6" t="n">
         <v>45149</v>
       </c>
       <c r="E51" t="n">
@@ -5251,7 +5098,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D52" s="8" t="n">
+      <c r="D52" s="6" t="n">
         <v>45170</v>
       </c>
       <c r="E52" t="n">
@@ -5322,7 +5169,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D53" s="8" t="n">
+      <c r="D53" s="6" t="n">
         <v>45170</v>
       </c>
       <c r="E53" t="n">
@@ -5399,7 +5246,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D54" s="8" t="n">
+      <c r="D54" s="6" t="n">
         <v>45175</v>
       </c>
       <c r="E54" t="n">
@@ -5458,7 +5305,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D55" s="8" t="n">
+      <c r="D55" s="6" t="n">
         <v>45175</v>
       </c>
       <c r="E55" t="n">
@@ -5523,7 +5370,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D56" s="8" t="n">
+      <c r="D56" s="6" t="n">
         <v>45255</v>
       </c>
       <c r="E56" t="n">
@@ -5597,7 +5444,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D57" s="8" t="n">
+      <c r="D57" s="6" t="n">
         <v>45255</v>
       </c>
       <c r="E57" t="n">
@@ -5668,7 +5515,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D58" s="8" t="n">
+      <c r="D58" s="6" t="n">
         <v>45255</v>
       </c>
       <c r="E58" t="n">
@@ -5748,7 +5595,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D59" s="8" t="n">
+      <c r="D59" s="6" t="n">
         <v>45275</v>
       </c>
       <c r="E59" t="n">
@@ -5819,7 +5666,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D60" s="8" t="n">
+      <c r="D60" s="6" t="n">
         <v>45275</v>
       </c>
       <c r="E60" t="n">
@@ -5896,7 +5743,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D61" s="8" t="n">
+      <c r="D61" s="6" t="n">
         <v>45278</v>
       </c>
       <c r="E61" t="n">
@@ -5973,7 +5820,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D62" s="8" t="n">
+      <c r="D62" s="6" t="n">
         <v>45278</v>
       </c>
       <c r="E62" t="n">
@@ -6050,7 +5897,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D63" s="8" t="n">
+      <c r="D63" s="6" t="n">
         <v>45280</v>
       </c>
       <c r="E63" t="n">
@@ -6121,7 +5968,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D64" s="8" t="n">
+      <c r="D64" s="6" t="n">
         <v>45315</v>
       </c>
       <c r="E64" t="n">
@@ -6192,7 +6039,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D65" s="8" t="n">
+      <c r="D65" s="6" t="n">
         <v>45352</v>
       </c>
       <c r="E65" t="n">
@@ -6263,7 +6110,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D66" s="8" t="n">
+      <c r="D66" s="6" t="n">
         <v>45357</v>
       </c>
       <c r="E66" t="n">
@@ -6334,7 +6181,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D67" s="8" t="n">
+      <c r="D67" s="6" t="n">
         <v>45369</v>
       </c>
       <c r="E67" t="n">
@@ -6405,7 +6252,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D68" s="8" t="n">
+      <c r="D68" s="6" t="n">
         <v>45376</v>
       </c>
       <c r="E68" t="n">
@@ -6476,7 +6323,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D69" s="8" t="n">
+      <c r="D69" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E69" t="n">
@@ -6547,7 +6394,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D70" s="8" t="n">
+      <c r="D70" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E70" t="n">
@@ -6618,7 +6465,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D71" s="8" t="n">
+      <c r="D71" s="6" t="n">
         <v>45381</v>
       </c>
       <c r="E71" t="n">
@@ -6677,7 +6524,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D72" s="8" t="n">
+      <c r="D72" s="6" t="n">
         <v>45383</v>
       </c>
       <c r="E72" t="n">
@@ -6748,7 +6595,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D73" s="8" t="n">
+      <c r="D73" s="6" t="n">
         <v>45433</v>
       </c>
       <c r="E73" t="n">
@@ -6819,7 +6666,7 @@
           <t>Truck Restriction</t>
         </is>
       </c>
-      <c r="D74" s="8" t="n">
+      <c r="D74" s="6" t="n">
         <v>45433</v>
       </c>
       <c r="E74" t="n">
@@ -6890,7 +6737,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D75" s="8" t="n">
+      <c r="D75" s="6" t="n">
         <v>45170</v>
       </c>
       <c r="E75" t="n">
@@ -6961,7 +6808,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D76" s="8" t="n">
+      <c r="D76" s="6" t="n">
         <v>45170</v>
       </c>
       <c r="E76" t="n">
@@ -7041,7 +6888,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D77" s="8" t="n">
+      <c r="D77" s="6" t="n">
         <v>45175</v>
       </c>
       <c r="E77" t="n">
@@ -7112,7 +6959,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D78" s="8" t="n">
+      <c r="D78" s="6" t="n">
         <v>45182</v>
       </c>
       <c r="E78" t="n">
@@ -7192,7 +7039,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D79" s="8" t="n">
+      <c r="D79" s="6" t="n">
         <v>45199</v>
       </c>
       <c r="E79" t="n">
@@ -7257,7 +7104,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D80" s="8" t="n">
+      <c r="D80" s="6" t="n">
         <v>45202</v>
       </c>
       <c r="E80" t="n">
@@ -7337,7 +7184,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D81" s="8" t="n">
+      <c r="D81" s="6" t="n">
         <v>45232</v>
       </c>
       <c r="E81" t="n">
@@ -7417,7 +7264,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D82" s="8" t="n">
+      <c r="D82" s="6" t="n">
         <v>45255</v>
       </c>
       <c r="E82" t="n">
@@ -7494,7 +7341,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D83" s="8" t="n">
+      <c r="D83" s="6" t="n">
         <v>45255</v>
       </c>
       <c r="E83" t="n">
@@ -7574,7 +7421,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D84" s="8" t="n">
+      <c r="D84" s="6" t="n">
         <v>45305</v>
       </c>
       <c r="E84" t="n">
@@ -7648,7 +7495,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D85" s="8" t="n">
+      <c r="D85" s="6" t="n">
         <v>45305</v>
       </c>
       <c r="E85" t="n">
@@ -7722,7 +7569,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D86" s="8" t="n">
+      <c r="D86" s="6" t="n">
         <v>45305</v>
       </c>
       <c r="E86" t="n">
@@ -7796,7 +7643,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D87" s="8" t="n">
+      <c r="D87" s="6" t="n">
         <v>45305</v>
       </c>
       <c r="E87" t="n">
@@ -7870,7 +7717,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D88" s="8" t="n">
+      <c r="D88" s="6" t="n">
         <v>45305</v>
       </c>
       <c r="E88" t="n">
@@ -7941,7 +7788,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D89" s="8" t="n">
+      <c r="D89" s="6" t="n">
         <v>45317</v>
       </c>
       <c r="E89" t="n">
@@ -8012,7 +7859,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D90" s="8" t="n">
+      <c r="D90" s="6" t="n">
         <v>45357</v>
       </c>
       <c r="E90" t="n">
@@ -8083,7 +7930,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D91" s="8" t="n">
+      <c r="D91" s="6" t="n">
         <v>45357</v>
       </c>
       <c r="E91" t="n">
@@ -8160,7 +8007,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D92" s="8" t="n">
+      <c r="D92" s="6" t="n">
         <v>45365</v>
       </c>
       <c r="E92" t="n">
@@ -8234,7 +8081,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D93" s="8" t="n">
+      <c r="D93" s="6" t="n">
         <v>45367</v>
       </c>
       <c r="E93" t="n">
@@ -8305,7 +8152,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D94" s="8" t="n">
+      <c r="D94" s="6" t="n">
         <v>45368</v>
       </c>
       <c r="E94" t="n">
@@ -8385,7 +8232,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D95" s="8" t="n">
+      <c r="D95" s="6" t="n">
         <v>45368</v>
       </c>
       <c r="E95" t="n">
@@ -8459,7 +8306,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D96" s="8" t="n">
+      <c r="D96" s="6" t="n">
         <v>45368</v>
       </c>
       <c r="E96" t="n">
@@ -8533,7 +8380,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D97" s="8" t="n">
+      <c r="D97" s="6" t="n">
         <v>45371</v>
       </c>
       <c r="E97" t="n">
@@ -8613,7 +8460,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D98" s="8" t="n">
+      <c r="D98" s="6" t="n">
         <v>45377</v>
       </c>
       <c r="E98" t="n">
@@ -8684,7 +8531,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D99" s="8" t="n">
+      <c r="D99" s="6" t="n">
         <v>45379</v>
       </c>
       <c r="E99" t="n">
@@ -8755,7 +8602,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D100" s="8" t="n">
+      <c r="D100" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E100" t="n">
@@ -8835,7 +8682,7 @@
           <t>Truck Restriction</t>
         </is>
       </c>
-      <c r="D101" s="8" t="n">
+      <c r="D101" s="6" t="n">
         <v>45383</v>
       </c>
       <c r="E101" t="n">
@@ -8906,7 +8753,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D102" s="8" t="n">
+      <c r="D102" s="6" t="n">
         <v>45384</v>
       </c>
       <c r="E102" t="n">
@@ -8977,7 +8824,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D103" s="8" t="n">
+      <c r="D103" s="6" t="n">
         <v>45384</v>
       </c>
       <c r="E103" t="n">
@@ -9054,7 +8901,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D104" s="8" t="n">
+      <c r="D104" s="6" t="n">
         <v>45392</v>
       </c>
       <c r="E104" t="n">
@@ -9128,7 +8975,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D105" s="8" t="n">
+      <c r="D105" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E105" t="n">
@@ -9193,7 +9040,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D106" s="8" t="n">
+      <c r="D106" s="6" t="n">
         <v>45671</v>
       </c>
       <c r="E106" t="n">
@@ -9273,7 +9120,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D107" s="8" t="n">
+      <c r="D107" s="6" t="n">
         <v>45671</v>
       </c>
       <c r="E107" t="n">
@@ -9347,7 +9194,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D108" s="8" t="n">
+      <c r="D108" s="6" t="n">
         <v>45671</v>
       </c>
       <c r="E108" t="n">
@@ -9421,7 +9268,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D109" s="8" t="n">
+      <c r="D109" s="6" t="n">
         <v>45671</v>
       </c>
       <c r="E109" t="n">
@@ -9507,7 +9354,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D110" s="8" t="n">
+      <c r="D110" s="6" t="n">
         <v>45149</v>
       </c>
       <c r="E110" t="n">
@@ -9587,7 +9434,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D111" s="8" t="n">
+      <c r="D111" s="6" t="n">
         <v>45175</v>
       </c>
       <c r="E111" t="n">
@@ -9661,7 +9508,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D112" s="8" t="n">
+      <c r="D112" s="6" t="n">
         <v>45227</v>
       </c>
       <c r="E112" t="n">
@@ -9735,7 +9582,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D113" s="8" t="n">
+      <c r="D113" s="6" t="n">
         <v>45278</v>
       </c>
       <c r="E113" t="n">
@@ -9815,7 +9662,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D114" s="8" t="n">
+      <c r="D114" s="6" t="n">
         <v>45278</v>
       </c>
       <c r="E114" t="n">
@@ -9895,7 +9742,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D115" s="8" t="n">
+      <c r="D115" s="6" t="n">
         <v>45278</v>
       </c>
       <c r="E115" t="n">
@@ -9969,7 +9816,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D116" s="8" t="n">
+      <c r="D116" s="6" t="n">
         <v>45287</v>
       </c>
       <c r="E116" t="n">
@@ -10049,7 +9896,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D117" s="8" t="n">
+      <c r="D117" s="6" t="n">
         <v>45305</v>
       </c>
       <c r="E117" t="n">
@@ -10126,7 +9973,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D118" s="8" t="n">
+      <c r="D118" s="6" t="n">
         <v>45305</v>
       </c>
       <c r="E118" t="n">
@@ -10200,7 +10047,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D119" s="8" t="n">
+      <c r="D119" s="6" t="n">
         <v>45305</v>
       </c>
       <c r="E119" t="n">
@@ -10271,7 +10118,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D120" s="8" t="n">
+      <c r="D120" s="6" t="n">
         <v>45305</v>
       </c>
       <c r="E120" t="n">
@@ -10348,7 +10195,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D121" s="8" t="n">
+      <c r="D121" s="6" t="n">
         <v>45314</v>
       </c>
       <c r="E121" t="n">
@@ -10434,7 +10281,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D122" s="8" t="n">
+      <c r="D122" s="6" t="n">
         <v>45321</v>
       </c>
       <c r="E122" t="n">
@@ -10508,7 +10355,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D123" s="8" t="n">
+      <c r="D123" s="6" t="n">
         <v>45330</v>
       </c>
       <c r="E123" t="n">
@@ -10582,7 +10429,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D124" s="8" t="n">
+      <c r="D124" s="6" t="n">
         <v>45331</v>
       </c>
       <c r="E124" t="n">
@@ -10653,7 +10500,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D125" s="8" t="n">
+      <c r="D125" s="6" t="n">
         <v>45331</v>
       </c>
       <c r="E125" t="n">
@@ -10724,7 +10571,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D126" s="8" t="n">
+      <c r="D126" s="6" t="n">
         <v>45346</v>
       </c>
       <c r="E126" t="n">
@@ -10804,7 +10651,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D127" s="8" t="n">
+      <c r="D127" s="6" t="n">
         <v>45352</v>
       </c>
       <c r="E127" t="n">
@@ -10878,7 +10725,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D128" s="8" t="n">
+      <c r="D128" s="6" t="n">
         <v>45357</v>
       </c>
       <c r="E128" t="n">
@@ -10949,7 +10796,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D129" s="8" t="n">
+      <c r="D129" s="6" t="n">
         <v>45357</v>
       </c>
       <c r="E129" t="n">
@@ -11014,7 +10861,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D130" s="8" t="n">
+      <c r="D130" s="6" t="n">
         <v>45357</v>
       </c>
       <c r="E130" t="n">
@@ -11088,7 +10935,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D131" s="8" t="n">
+      <c r="D131" s="6" t="n">
         <v>45357</v>
       </c>
       <c r="E131" t="n">
@@ -11159,7 +11006,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D132" s="8" t="n">
+      <c r="D132" s="6" t="n">
         <v>45366</v>
       </c>
       <c r="E132" t="n">
@@ -11230,7 +11077,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D133" s="8" t="n">
+      <c r="D133" s="6" t="n">
         <v>45372</v>
       </c>
       <c r="E133" t="n">
@@ -11310,7 +11157,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D134" s="8" t="n">
+      <c r="D134" s="6" t="n">
         <v>45372</v>
       </c>
       <c r="E134" t="n">
@@ -11381,7 +11228,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D135" s="8" t="n">
+      <c r="D135" s="6" t="n">
         <v>45379</v>
       </c>
       <c r="E135" t="n">
@@ -11452,7 +11299,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D136" s="8" t="n">
+      <c r="D136" s="6" t="n">
         <v>45379</v>
       </c>
       <c r="E136" t="n">
@@ -11526,7 +11373,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D137" s="8" t="n">
+      <c r="D137" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E137" t="n">
@@ -11600,7 +11447,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D138" s="8" t="n">
+      <c r="D138" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E138" t="n">
@@ -11677,7 +11524,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D139" s="8" t="n">
+      <c r="D139" s="6" t="n">
         <v>45381</v>
       </c>
       <c r="E139" t="n">
@@ -11757,7 +11604,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D140" s="8" t="n">
+      <c r="D140" s="6" t="n">
         <v>45381</v>
       </c>
       <c r="E140" t="n">
@@ -11828,7 +11675,7 @@
           <t>Truck Restriction</t>
         </is>
       </c>
-      <c r="D141" s="8" t="n">
+      <c r="D141" s="6" t="n">
         <v>45383</v>
       </c>
       <c r="E141" t="n">
@@ -11902,7 +11749,7 @@
           <t>Truck Restriction</t>
         </is>
       </c>
-      <c r="D142" s="8" t="n">
+      <c r="D142" s="6" t="n">
         <v>45383</v>
       </c>
       <c r="E142" t="n">
@@ -11973,7 +11820,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D143" s="8" t="n">
+      <c r="D143" s="6" t="n">
         <v>45383</v>
       </c>
       <c r="E143" t="n">
@@ -12044,7 +11891,7 @@
           <t>Truck Restriction</t>
         </is>
       </c>
-      <c r="D144" s="8" t="n">
+      <c r="D144" s="6" t="n">
         <v>45383</v>
       </c>
       <c r="E144" t="n">
@@ -12115,7 +11962,7 @@
           <t>Truck Restriction</t>
         </is>
       </c>
-      <c r="D145" s="8" t="n">
+      <c r="D145" s="6" t="n">
         <v>45383</v>
       </c>
       <c r="E145" t="n">
@@ -12195,7 +12042,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D146" s="8" t="n">
+      <c r="D146" s="6" t="n">
         <v>45383</v>
       </c>
       <c r="E146" t="n">
@@ -12266,7 +12113,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D147" s="8" t="n">
+      <c r="D147" s="6" t="n">
         <v>45384</v>
       </c>
       <c r="E147" t="n">
@@ -12346,7 +12193,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D148" s="8" t="n">
+      <c r="D148" s="6" t="n">
         <v>45388</v>
       </c>
       <c r="E148" t="n">
@@ -12423,7 +12270,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D149" s="8" t="n">
+      <c r="D149" s="6" t="n">
         <v>45392</v>
       </c>
       <c r="E149" t="n">
@@ -12500,7 +12347,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D150" s="8" t="n">
+      <c r="D150" s="6" t="n">
         <v>45399</v>
       </c>
       <c r="E150" t="n">
@@ -12574,7 +12421,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D151" s="8" t="n">
+      <c r="D151" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E151" t="n">
@@ -12648,7 +12495,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D152" s="8" t="n">
+      <c r="D152" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E152" t="n">
@@ -12728,7 +12575,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D153" s="8" t="n">
+      <c r="D153" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E153" t="n">
@@ -12802,7 +12649,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D154" s="8" t="n">
+      <c r="D154" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E154" t="n">
@@ -12885,7 +12732,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D155" s="8" t="n">
+      <c r="D155" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E155" t="n">
@@ -12968,7 +12815,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D156" s="8" t="n">
+      <c r="D156" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E156" t="n">
@@ -13048,7 +12895,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D157" s="8" t="n">
+      <c r="D157" s="6" t="n">
         <v>45433</v>
       </c>
       <c r="E157" t="n">
@@ -13128,7 +12975,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D158" s="8" t="n">
+      <c r="D158" s="6" t="n">
         <v>45490</v>
       </c>
       <c r="E158" t="n">
@@ -13187,7 +13034,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D159" s="8" t="n">
+      <c r="D159" s="6" t="n">
         <v>45490</v>
       </c>
       <c r="E159" t="n">
@@ -13246,7 +13093,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D160" s="8" t="n">
+      <c r="D160" s="6" t="n">
         <v>45490</v>
       </c>
       <c r="E160" t="n">
@@ -13326,7 +13173,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D161" s="8" t="n">
+      <c r="D161" s="6" t="n">
         <v>45490</v>
       </c>
       <c r="E161" t="n">
@@ -13406,7 +13253,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D162" s="8" t="n">
+      <c r="D162" s="6" t="n">
         <v>45503</v>
       </c>
       <c r="E162" t="n">
@@ -13480,7 +13327,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D163" s="8" t="n">
+      <c r="D163" s="6" t="n">
         <v>45540</v>
       </c>
       <c r="E163" t="n">
@@ -13551,7 +13398,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D164" s="8" t="n">
+      <c r="D164" s="6" t="n">
         <v>45619</v>
       </c>
       <c r="E164" t="n">
@@ -13631,7 +13478,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D165" s="8" t="n">
+      <c r="D165" s="6" t="n">
         <v>45619</v>
       </c>
       <c r="E165" t="n">
@@ -13711,7 +13558,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D166" s="8" t="n">
+      <c r="D166" s="6" t="n">
         <v>45639</v>
       </c>
       <c r="E166" t="n">
@@ -13797,7 +13644,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D167" s="8" t="n">
+      <c r="D167" s="6" t="n">
         <v>45639</v>
       </c>
       <c r="E167" t="n">
@@ -13883,7 +13730,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D168" s="8" t="n">
+      <c r="D168" s="6" t="n">
         <v>45305</v>
       </c>
       <c r="E168" t="n">
@@ -13957,7 +13804,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D169" s="8" t="n">
+      <c r="D169" s="6" t="n">
         <v>45314</v>
       </c>
       <c r="E169" t="n">
@@ -14031,7 +13878,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D170" s="8" t="n">
+      <c r="D170" s="6" t="n">
         <v>45314</v>
       </c>
       <c r="E170" t="n">
@@ -14111,7 +13958,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D171" s="8" t="n">
+      <c r="D171" s="6" t="n">
         <v>45330</v>
       </c>
       <c r="E171" t="n">
@@ -14191,7 +14038,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D172" s="8" t="n">
+      <c r="D172" s="6" t="n">
         <v>45367</v>
       </c>
       <c r="E172" t="n">
@@ -14265,7 +14112,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D173" s="8" t="n">
+      <c r="D173" s="6" t="n">
         <v>45368</v>
       </c>
       <c r="E173" t="n">
@@ -14339,7 +14186,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D174" s="8" t="n">
+      <c r="D174" s="6" t="n">
         <v>45372</v>
       </c>
       <c r="E174" t="n">
@@ -14419,7 +14266,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D175" s="8" t="n">
+      <c r="D175" s="6" t="n">
         <v>45376</v>
       </c>
       <c r="E175" t="n">
@@ -14499,7 +14346,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D176" s="8" t="n">
+      <c r="D176" s="6" t="n">
         <v>45376</v>
       </c>
       <c r="E176" t="n">
@@ -14579,7 +14426,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D177" s="8" t="n">
+      <c r="D177" s="6" t="n">
         <v>45378</v>
       </c>
       <c r="E177" t="n">
@@ -14653,7 +14500,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D178" s="8" t="n">
+      <c r="D178" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E178" t="n">
@@ -14733,7 +14580,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D179" s="8" t="n">
+      <c r="D179" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E179" t="n">
@@ -14813,7 +14660,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D180" s="8" t="n">
+      <c r="D180" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E180" t="n">
@@ -14887,7 +14734,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D181" s="8" t="n">
+      <c r="D181" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E181" t="n">
@@ -14967,7 +14814,7 @@
           <t>Truck Restriction</t>
         </is>
       </c>
-      <c r="D182" s="8" t="n">
+      <c r="D182" s="6" t="n">
         <v>45383</v>
       </c>
       <c r="E182" t="n">
@@ -15041,7 +14888,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D183" s="8" t="n">
+      <c r="D183" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E183" t="n">
@@ -15115,7 +14962,7 @@
           <t>Truck Restriction</t>
         </is>
       </c>
-      <c r="D184" s="8" t="n">
+      <c r="D184" s="6" t="n">
         <v>45433</v>
       </c>
       <c r="E184" t="n">
@@ -15189,7 +15036,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D185" s="8" t="n">
+      <c r="D185" s="6" t="n">
         <v>45149</v>
       </c>
       <c r="E185" t="n">
@@ -15269,7 +15116,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D186" s="8" t="n">
+      <c r="D186" s="6" t="n">
         <v>45149</v>
       </c>
       <c r="E186" t="n">
@@ -15343,7 +15190,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D187" s="8" t="n">
+      <c r="D187" s="6" t="n">
         <v>45170</v>
       </c>
       <c r="E187" t="n">
@@ -15420,7 +15267,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D188" s="8" t="n">
+      <c r="D188" s="6" t="n">
         <v>45175</v>
       </c>
       <c r="E188" t="n">
@@ -15500,7 +15347,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D189" s="8" t="n">
+      <c r="D189" s="6" t="n">
         <v>45198</v>
       </c>
       <c r="E189" t="n">
@@ -15580,7 +15427,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D190" s="8" t="n">
+      <c r="D190" s="6" t="n">
         <v>45231</v>
       </c>
       <c r="E190" t="n">
@@ -15660,7 +15507,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D191" s="8" t="n">
+      <c r="D191" s="6" t="n">
         <v>45232</v>
       </c>
       <c r="E191" t="n">
@@ -15734,7 +15581,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D192" s="8" t="n">
+      <c r="D192" s="6" t="n">
         <v>45255</v>
       </c>
       <c r="E192" t="n">
@@ -15808,7 +15655,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D193" s="8" t="n">
+      <c r="D193" s="6" t="n">
         <v>45255</v>
       </c>
       <c r="E193" t="n">
@@ -15888,7 +15735,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D194" s="8" t="n">
+      <c r="D194" s="6" t="n">
         <v>45255</v>
       </c>
       <c r="E194" t="n">
@@ -15968,7 +15815,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D195" s="8" t="n">
+      <c r="D195" s="6" t="n">
         <v>45255</v>
       </c>
       <c r="E195" t="n">
@@ -16048,7 +15895,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D196" s="8" t="n">
+      <c r="D196" s="6" t="n">
         <v>45255</v>
       </c>
       <c r="E196" t="n">
@@ -16122,7 +15969,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D197" s="8" t="n">
+      <c r="D197" s="6" t="n">
         <v>45278</v>
       </c>
       <c r="E197" t="n">
@@ -16202,7 +16049,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D198" s="8" t="n">
+      <c r="D198" s="6" t="n">
         <v>45290</v>
       </c>
       <c r="E198" t="n">
@@ -16273,7 +16120,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D199" s="8" t="n">
+      <c r="D199" s="6" t="n">
         <v>45290</v>
       </c>
       <c r="E199" t="n">
@@ -16347,7 +16194,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D200" s="8" t="n">
+      <c r="D200" s="6" t="n">
         <v>45290</v>
       </c>
       <c r="E200" t="n">
@@ -16433,7 +16280,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D201" s="8" t="n">
+      <c r="D201" s="6" t="n">
         <v>45290</v>
       </c>
       <c r="E201" t="n">
@@ -16513,7 +16360,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D202" s="8" t="n">
+      <c r="D202" s="6" t="n">
         <v>45305</v>
       </c>
       <c r="E202" t="n">
@@ -16584,7 +16431,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D203" s="8" t="n">
+      <c r="D203" s="6" t="n">
         <v>45305</v>
       </c>
       <c r="E203" t="n">
@@ -16658,7 +16505,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D204" s="8" t="n">
+      <c r="D204" s="6" t="n">
         <v>45314</v>
       </c>
       <c r="E204" t="n">
@@ -16744,7 +16591,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D205" s="8" t="n">
+      <c r="D205" s="6" t="n">
         <v>45352</v>
       </c>
       <c r="E205" t="n">
@@ -16818,7 +16665,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D206" s="8" t="n">
+      <c r="D206" s="6" t="n">
         <v>45352</v>
       </c>
       <c r="E206" t="n">
@@ -16892,7 +16739,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D207" s="8" t="n">
+      <c r="D207" s="6" t="n">
         <v>45357</v>
       </c>
       <c r="E207" t="n">
@@ -16966,7 +16813,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D208" s="8" t="n">
+      <c r="D208" s="6" t="n">
         <v>45357</v>
       </c>
       <c r="E208" t="n">
@@ -17040,7 +16887,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D209" s="8" t="n">
+      <c r="D209" s="6" t="n">
         <v>45365</v>
       </c>
       <c r="E209" t="n">
@@ -17120,7 +16967,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D210" s="8" t="n">
+      <c r="D210" s="6" t="n">
         <v>45365</v>
       </c>
       <c r="E210" t="n">
@@ -17197,7 +17044,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D211" s="8" t="n">
+      <c r="D211" s="6" t="n">
         <v>45368</v>
       </c>
       <c r="E211" t="n">
@@ -17277,7 +17124,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D212" s="8" t="n">
+      <c r="D212" s="6" t="n">
         <v>45368</v>
       </c>
       <c r="E212" t="n">
@@ -17354,7 +17201,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D213" s="8" t="n">
+      <c r="D213" s="6" t="n">
         <v>45368</v>
       </c>
       <c r="E213" t="n">
@@ -17425,7 +17272,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D214" s="8" t="n">
+      <c r="D214" s="6" t="n">
         <v>45371</v>
       </c>
       <c r="E214" t="n">
@@ -17499,7 +17346,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D215" s="8" t="n">
+      <c r="D215" s="6" t="n">
         <v>45371</v>
       </c>
       <c r="E215" t="n">
@@ -17573,7 +17420,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D216" s="8" t="n">
+      <c r="D216" s="6" t="n">
         <v>45371</v>
       </c>
       <c r="E216" t="n">
@@ -17647,7 +17494,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D217" s="8" t="n">
+      <c r="D217" s="6" t="n">
         <v>45371</v>
       </c>
       <c r="E217" t="n">
@@ -17721,7 +17568,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D218" s="8" t="n">
+      <c r="D218" s="6" t="n">
         <v>45371</v>
       </c>
       <c r="E218" t="n">
@@ -17792,7 +17639,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D219" s="8" t="n">
+      <c r="D219" s="6" t="n">
         <v>45376</v>
       </c>
       <c r="E219" t="n">
@@ -17866,7 +17713,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D220" s="8" t="n">
+      <c r="D220" s="6" t="n">
         <v>45377</v>
       </c>
       <c r="E220" t="n">
@@ -17931,7 +17778,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D221" s="8" t="n">
+      <c r="D221" s="6" t="n">
         <v>45378</v>
       </c>
       <c r="E221" t="n">
@@ -18002,7 +17849,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D222" s="8" t="n">
+      <c r="D222" s="6" t="n">
         <v>45378</v>
       </c>
       <c r="E222" t="n">
@@ -18076,7 +17923,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D223" s="8" t="n">
+      <c r="D223" s="6" t="n">
         <v>45379</v>
       </c>
       <c r="E223" t="n">
@@ -18150,7 +17997,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D224" s="8" t="n">
+      <c r="D224" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E224" t="n">
@@ -18227,7 +18074,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D225" s="8" t="n">
+      <c r="D225" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E225" t="n">
@@ -18304,7 +18151,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D226" s="8" t="n">
+      <c r="D226" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E226" t="n">
@@ -18375,7 +18222,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D227" s="8" t="n">
+      <c r="D227" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E227" t="n">
@@ -18446,7 +18293,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D228" s="8" t="n">
+      <c r="D228" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E228" t="n">
@@ -18520,7 +18367,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D229" s="8" t="n">
+      <c r="D229" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E229" t="n">
@@ -18600,7 +18447,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D230" s="8" t="n">
+      <c r="D230" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E230" t="n">
@@ -18680,7 +18527,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D231" s="8" t="n">
+      <c r="D231" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E231" t="n">
@@ -18760,7 +18607,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D232" s="8" t="n">
+      <c r="D232" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E232" t="n">
@@ -18840,7 +18687,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D233" s="8" t="n">
+      <c r="D233" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E233" t="n">
@@ -18926,7 +18773,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D234" s="8" t="n">
+      <c r="D234" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E234" t="n">
@@ -19000,7 +18847,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D235" s="8" t="n">
+      <c r="D235" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E235" t="n">
@@ -19074,7 +18921,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D236" s="8" t="n">
+      <c r="D236" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E236" t="n">
@@ -19148,7 +18995,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D237" s="8" t="n">
+      <c r="D237" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E237" t="n">
@@ -19219,7 +19066,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D238" s="8" t="n">
+      <c r="D238" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E238" t="n">
@@ -19305,7 +19152,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D239" s="8" t="n">
+      <c r="D239" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E239" t="n">
@@ -19376,7 +19223,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D240" s="8" t="n">
+      <c r="D240" s="6" t="n">
         <v>45381</v>
       </c>
       <c r="E240" t="n">
@@ -19447,7 +19294,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D241" s="8" t="n">
+      <c r="D241" s="6" t="n">
         <v>45381</v>
       </c>
       <c r="E241" t="n">
@@ -19527,7 +19374,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D242" s="8" t="n">
+      <c r="D242" s="6" t="n">
         <v>45381</v>
       </c>
       <c r="E242" t="n">
@@ -19598,7 +19445,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D243" s="8" t="n">
+      <c r="D243" s="6" t="n">
         <v>45386</v>
       </c>
       <c r="E243" t="n">
@@ -19672,7 +19519,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D244" s="8" t="n">
+      <c r="D244" s="6" t="n">
         <v>45392</v>
       </c>
       <c r="E244" t="n">
@@ -19758,7 +19605,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D245" s="8" t="n">
+      <c r="D245" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E245" t="n">
@@ -19829,7 +19676,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D246" s="8" t="n">
+      <c r="D246" s="6" t="n">
         <v>45408</v>
       </c>
       <c r="E246" t="n">
@@ -19909,7 +19756,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D247" s="8" t="n">
+      <c r="D247" s="6" t="n">
         <v>45484</v>
       </c>
       <c r="E247" t="n">
@@ -19983,7 +19830,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D248" s="8" t="n">
+      <c r="D248" s="6" t="n">
         <v>45484</v>
       </c>
       <c r="E248" t="n">
@@ -20063,7 +19910,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D249" s="8" t="n">
+      <c r="D249" s="6" t="n">
         <v>45500</v>
       </c>
       <c r="E249" t="n">
@@ -20137,7 +19984,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D250" s="8" t="n">
+      <c r="D250" s="6" t="n">
         <v>45170</v>
       </c>
       <c r="E250" t="n">
@@ -20211,7 +20058,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D251" s="8" t="n">
+      <c r="D251" s="6" t="n">
         <v>45255</v>
       </c>
       <c r="E251" t="n">
@@ -20291,7 +20138,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D252" s="8" t="n">
+      <c r="D252" s="6" t="n">
         <v>45255</v>
       </c>
       <c r="E252" t="n">
@@ -20371,7 +20218,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D253" s="8" t="n">
+      <c r="D253" s="6" t="n">
         <v>45282</v>
       </c>
       <c r="E253" t="n">
@@ -20442,7 +20289,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D254" s="8" t="n">
+      <c r="D254" s="6" t="n">
         <v>45282</v>
       </c>
       <c r="E254" t="n">
@@ -20516,7 +20363,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D255" s="8" t="n">
+      <c r="D255" s="6" t="n">
         <v>45290</v>
       </c>
       <c r="E255" t="n">
@@ -20590,7 +20437,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D256" s="8" t="n">
+      <c r="D256" s="6" t="n">
         <v>45290</v>
       </c>
       <c r="E256" t="n">
@@ -20664,7 +20511,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D257" s="8" t="n">
+      <c r="D257" s="6" t="n">
         <v>45302</v>
       </c>
       <c r="E257" t="n">
@@ -20741,7 +20588,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D258" s="8" t="n">
+      <c r="D258" s="6" t="n">
         <v>45314</v>
       </c>
       <c r="E258" t="n">
@@ -20818,7 +20665,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D259" s="8" t="n">
+      <c r="D259" s="6" t="n">
         <v>45322</v>
       </c>
       <c r="E259" t="n">
@@ -20892,7 +20739,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D260" s="8" t="n">
+      <c r="D260" s="6" t="n">
         <v>45331</v>
       </c>
       <c r="E260" t="n">
@@ -20966,7 +20813,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D261" s="8" t="n">
+      <c r="D261" s="6" t="n">
         <v>45334</v>
       </c>
       <c r="E261" t="n">
@@ -21052,7 +20899,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D262" s="8" t="n">
+      <c r="D262" s="6" t="n">
         <v>45365</v>
       </c>
       <c r="E262" t="n">
@@ -21117,7 +20964,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D263" s="8" t="n">
+      <c r="D263" s="6" t="n">
         <v>45368</v>
       </c>
       <c r="E263" t="n">
@@ -21194,7 +21041,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D264" s="8" t="n">
+      <c r="D264" s="6" t="n">
         <v>45368</v>
       </c>
       <c r="E264" t="n">
@@ -21268,7 +21115,7 @@
           <t>Stop Sign</t>
         </is>
       </c>
-      <c r="D265" s="8" t="n">
+      <c r="D265" s="6" t="n">
         <v>45368</v>
       </c>
       <c r="E265" t="n">
@@ -21339,7 +21186,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D266" s="8" t="n">
+      <c r="D266" s="6" t="n">
         <v>45371</v>
       </c>
       <c r="E266" t="n">
@@ -21425,7 +21272,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D267" s="8" t="n">
+      <c r="D267" s="6" t="n">
         <v>45376</v>
       </c>
       <c r="E267" t="n">
@@ -21496,7 +21343,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D268" s="8" t="n">
+      <c r="D268" s="6" t="n">
         <v>45377</v>
       </c>
       <c r="E268" t="n">
@@ -21570,7 +21417,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D269" s="8" t="n">
+      <c r="D269" s="6" t="n">
         <v>45379</v>
       </c>
       <c r="E269" t="n">
@@ -21641,7 +21488,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D270" s="8" t="n">
+      <c r="D270" s="6" t="n">
         <v>45379</v>
       </c>
       <c r="E270" t="n">
@@ -21706,7 +21553,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D271" s="8" t="n">
+      <c r="D271" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E271" t="n">
@@ -21780,7 +21627,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D272" s="8" t="n">
+      <c r="D272" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E272" t="n">
@@ -21854,7 +21701,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D273" s="8" t="n">
+      <c r="D273" s="6" t="n">
         <v>45380</v>
       </c>
       <c r="E273" t="n">
@@ -21925,7 +21772,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D274" s="8" t="n">
+      <c r="D274" s="6" t="n">
         <v>45381</v>
       </c>
       <c r="E274" t="n">
@@ -21999,7 +21846,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D275" s="8" t="n">
+      <c r="D275" s="6" t="n">
         <v>45381</v>
       </c>
       <c r="E275" t="n">
@@ -22079,7 +21926,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D276" s="8" t="n">
+      <c r="D276" s="6" t="n">
         <v>45381</v>
       </c>
       <c r="E276" t="n">
@@ -22150,7 +21997,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D277" s="8" t="n">
+      <c r="D277" s="6" t="n">
         <v>45381</v>
       </c>
       <c r="E277" t="n">
@@ -22224,7 +22071,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D278" s="8" t="n">
+      <c r="D278" s="6" t="n">
         <v>45381</v>
       </c>
       <c r="E278" t="n">
@@ -22295,7 +22142,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D279" s="8" t="n">
+      <c r="D279" s="6" t="n">
         <v>45384</v>
       </c>
       <c r="E279" t="n">
@@ -22369,7 +22216,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D280" s="8" t="n">
+      <c r="D280" s="6" t="n">
         <v>45555</v>
       </c>
       <c r="E280" t="n">
@@ -22440,7 +22287,7 @@
           <t>Speed</t>
         </is>
       </c>
-      <c r="D281" s="8" t="n">
+      <c r="D281" s="6" t="n">
         <v>45555</v>
       </c>
       <c r="E281" t="n">
@@ -22514,7 +22361,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D282" s="8" t="n">
+      <c r="D282" s="6" t="n">
         <v>45619</v>
       </c>
       <c r="E282" t="n">
@@ -22600,7 +22447,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D283" s="8" t="n">
+      <c r="D283" s="6" t="n">
         <v>45619</v>
       </c>
       <c r="E283" t="n">
@@ -22677,7 +22524,7 @@
           <t>Red Light</t>
         </is>
       </c>
-      <c r="D284" s="8" t="n">
+      <c r="D284" s="6" t="n">
         <v>45642</v>
       </c>
       <c r="E284" t="n">
@@ -22743,7 +22590,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22761,7 +22608,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Placebo test — install dates shifted back 1 year</t>
         </is>
@@ -22776,32 +22623,32 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Camera Type</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Outcome</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Real DiD</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Placebo DiD</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Corrected DiD (Real - Placebo)</t>
         </is>
@@ -23176,154 +23023,6 @@
       <c r="C23" t="inlineStr">
         <is>
           <t>Fatal only</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>DC Traffic Camera Impact Analysis — Methodology</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="10" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>DATA</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>Crash data: DDOT Crashes in DC dataset. 75,400 geocoded crashes, 2021–2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>Camera data: DDOT Automated Traffic Enforcement dataset. 283 eligible cameras.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>Buffer: 200m radius around each camera using geopy.distance for real-world distance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>Windows: 365 days before install vs 365 days after (install day excluded).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>DiD: (nearby % change) minus (citywide % change) over the same windows.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>VALIDITY CHECK</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>Placebo: each camera's install date shifted back 1 year. If the cameras cause the</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>effect, the placebo DiD should be close to zero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>LIMITATIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>1. Cameras are placed where crashes are elevated — regression to mean is a risk.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>2. 200m is a straight-line proxy, not a street-network distance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>3. Camera installs may coincide with other street changes (signs, paint, bollards).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>4. START_DATE is assumed to mean active enforcement; warning periods dilute the effect.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>5. Fatal/serious per-type counts are too sparse for confident claims.</t>
         </is>
       </c>
     </row>

</xml_diff>